<commit_message>
adding forcenew attributes to the site
</commit_message>
<xml_diff>
--- a/scripts/templates/cx-as-code-spreadsheet-template.xlsx
+++ b/scripts/templates/cx-as-code-spreadsheet-template.xlsx
@@ -1,56 +1,52 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ascheble/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8076B3B-A0D9-3942-A179-08CFA0AF627B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{166D1F10-E3AB-E94C-B675-684CCFA97A59}"/>
+    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680"/>
   </bookViews>
   <sheets>
-    <sheet name="resources" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="resources" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">resources!$A$1:$J$124</definedName>
+    <definedName name="_xlnm._FilterDatabase">resources!$A$1:$J$124</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="246">
   <si>
+    <t>GUI Menu Path</t>
+  </si>
+  <si>
     <t>CX as Code Resource Type</t>
   </si>
   <si>
     <t>Division-aware</t>
   </si>
   <si>
-    <t>Possible Dependencies</t>
+    <t>Dependencies</t>
+  </si>
+  <si>
+    <t>In/out of scope</t>
+  </si>
+  <si>
+    <t>Shared?</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Repo/Project/Folder</t>
+  </si>
+  <si>
+    <t>Transform type</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
   <si>
     <t>User Management &gt; ACD Skills and Languages &gt; Languages</t>
@@ -759,61 +755,47 @@
   </si>
   <si>
     <t>genesyscloud_webdeployments_deployment</t>
-  </si>
-  <si>
-    <t>GUI Menu Path</t>
-  </si>
-  <si>
-    <t>Repo/Project/Folder</t>
-  </si>
-  <si>
-    <t>Transform type</t>
-  </si>
-  <si>
-    <t>Shared?</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>In/out of scope</t>
-  </si>
-  <si>
-    <t>Notes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -844,13 +826,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1164,2269 +1146,2268 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444CE756-FC6B-BB41-9CFA-B458F0085971}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J124"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="73.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="67" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="11" max="11" width="2" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D16">
         <v>3</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>2</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C22" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D24">
         <v>1</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D27">
         <v>8</v>
       </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C30" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>13</v>
       </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D32">
         <v>3</v>
       </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C33" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C35" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D36">
         <v>1</v>
       </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D37">
         <v>3</v>
       </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C38" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D39">
         <v>2</v>
       </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D40">
         <v>0</v>
       </c>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D41">
         <v>3</v>
       </c>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D42">
         <v>2</v>
       </c>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B43" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D43">
         <v>2</v>
       </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C44" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D44">
         <v>2</v>
       </c>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C45" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D45">
         <v>0</v>
       </c>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D46">
         <v>0</v>
       </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C47" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D47">
         <v>1</v>
       </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C48" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C49" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C50" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D50">
         <v>0</v>
       </c>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C51" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D51">
         <v>0</v>
       </c>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C52" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C53" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D53">
         <v>0</v>
       </c>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C54" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D54">
         <v>0</v>
       </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B55" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C55" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D55">
         <v>0</v>
       </c>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B56" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C56" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D56">
         <v>2</v>
       </c>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="C57" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D57">
         <v>0</v>
       </c>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B58" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B59" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C59" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D59">
         <v>0</v>
       </c>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B60" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C60" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D60">
         <v>0</v>
       </c>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C61" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D61">
         <v>0</v>
       </c>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B62" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D62">
         <v>0</v>
       </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C63" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D63">
         <v>0</v>
       </c>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C64" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D64">
         <v>1</v>
       </c>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B65" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C65" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D65">
         <v>1</v>
       </c>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="5"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B66" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C66" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D66">
         <v>2</v>
       </c>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B67" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C67" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D67">
         <v>5</v>
       </c>
-      <c r="E67" s="4"/>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C68" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D68">
         <v>0</v>
       </c>
-      <c r="E68" s="4"/>
-      <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B69" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C69" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D69">
         <v>0</v>
       </c>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B70" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C70" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D71">
         <v>0</v>
       </c>
-      <c r="E71" s="4"/>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B72" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C72" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D72">
         <v>0</v>
       </c>
-      <c r="E72" s="4"/>
-      <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B73" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C73" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D73">
         <v>0</v>
       </c>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="5"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C74" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D74">
         <v>1</v>
       </c>
-      <c r="E74" s="4"/>
-      <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B75" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C75" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D75">
         <v>1</v>
       </c>
-      <c r="E75" s="4"/>
-      <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
-      <c r="H75" s="4"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B76" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C76" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D76">
         <v>2</v>
       </c>
-      <c r="E76" s="4"/>
-      <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
-      <c r="H76" s="4"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B77" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C77" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D77">
         <v>0</v>
       </c>
-      <c r="E77" s="4"/>
-      <c r="F77" s="4"/>
-      <c r="G77" s="4"/>
-      <c r="H77" s="4"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5"/>
+      <c r="H77" s="5"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B78" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C78" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D78">
         <v>1</v>
       </c>
-      <c r="E78" s="4"/>
-      <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
-      <c r="H78" s="4"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5"/>
+      <c r="H78" s="5"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B79" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C79" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D79">
         <v>3</v>
       </c>
-      <c r="E79" s="4"/>
-      <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B80" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C80" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D80">
         <v>0</v>
       </c>
-      <c r="E80" s="4"/>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B81" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C81" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D81">
         <v>1</v>
       </c>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
-      <c r="H81" s="4"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B82" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C82" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D82">
         <v>0</v>
       </c>
-      <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
-      <c r="G82" s="4"/>
-      <c r="H82" s="4"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B83" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C83" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D83">
         <v>0</v>
       </c>
-      <c r="E83" s="4"/>
-      <c r="F83" s="4"/>
-      <c r="G83" s="4"/>
-      <c r="H83" s="4"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B84" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C84" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D84">
         <v>1</v>
       </c>
-      <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
-      <c r="G84" s="4"/>
-      <c r="H84" s="4"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B85" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C85" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D85">
         <v>11</v>
       </c>
-      <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
-      <c r="H85" s="4"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B86" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C86" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D86">
         <v>5</v>
       </c>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-      <c r="H86" s="4"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5"/>
+      <c r="H86" s="5"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B87" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C87" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D87">
         <v>2</v>
       </c>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
-      <c r="H87" s="4"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
+      <c r="H87" s="5"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B88" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C88" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D88">
         <v>2</v>
       </c>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
-      <c r="G88" s="4"/>
-      <c r="H88" s="4"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="5"/>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B89" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C89" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D89">
         <v>2</v>
       </c>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
-      <c r="H89" s="4"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B90" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C90" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D90">
         <v>1</v>
       </c>
-      <c r="E90" s="4"/>
-      <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
-      <c r="H90" s="4"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B91" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C91" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D91">
         <v>1</v>
       </c>
-      <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
-      <c r="H91" s="4"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B92" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C92" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D92">
         <v>0</v>
       </c>
-      <c r="E92" s="4"/>
-      <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
-      <c r="H92" s="4"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B93" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C93" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D93">
         <v>9</v>
       </c>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
-      <c r="H93" s="4"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B94" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C94" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D94">
         <v>4</v>
       </c>
-      <c r="E94" s="4"/>
-      <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
-      <c r="H94" s="4"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B95" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C95" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D95">
         <v>1</v>
       </c>
-      <c r="E95" s="4"/>
-      <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
-      <c r="H95" s="4"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B96" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C96" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D96">
         <v>0</v>
       </c>
-      <c r="E96" s="4"/>
-      <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
-      <c r="H96" s="4"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B97" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C97" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D97">
         <v>1</v>
       </c>
-      <c r="E97" s="4"/>
-      <c r="F97" s="4"/>
-      <c r="G97" s="4"/>
-      <c r="H97" s="4"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B98" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C98" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D98">
         <v>1</v>
       </c>
-      <c r="E98" s="4"/>
-      <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
-      <c r="H98" s="4"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5"/>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B99" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C99" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D99">
         <v>2</v>
       </c>
-      <c r="E99" s="4"/>
-      <c r="F99" s="4"/>
-      <c r="G99" s="4"/>
-      <c r="H99" s="4"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B100" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C100" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D100">
         <v>1</v>
       </c>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
-      <c r="H100" s="4"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5"/>
+      <c r="H100" s="5"/>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B101" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C101" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D101">
         <v>5</v>
       </c>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
-      <c r="H101" s="4"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
+      <c r="G101" s="5"/>
+      <c r="H101" s="5"/>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B102" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C102" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D102">
         <v>0</v>
       </c>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
-      <c r="H102" s="4"/>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E102" s="5"/>
+      <c r="F102" s="5"/>
+      <c r="G102" s="5"/>
+      <c r="H102" s="5"/>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B103" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C103" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D103">
         <v>0</v>
       </c>
-      <c r="E103" s="4"/>
-      <c r="F103" s="4"/>
-      <c r="G103" s="4"/>
-      <c r="H103" s="4"/>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E103" s="5"/>
+      <c r="F103" s="5"/>
+      <c r="G103" s="5"/>
+      <c r="H103" s="5"/>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B104" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C104" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D104">
         <v>0</v>
       </c>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
-      <c r="H104" s="4"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E104" s="5"/>
+      <c r="F104" s="5"/>
+      <c r="G104" s="5"/>
+      <c r="H104" s="5"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B105" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C105" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D105">
         <v>0</v>
       </c>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
-      <c r="G105" s="4"/>
-      <c r="H105" s="4"/>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
+      <c r="G105" s="5"/>
+      <c r="H105" s="5"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="B106" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C106" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D106">
         <v>1</v>
       </c>
-      <c r="E106" s="4"/>
-      <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
-      <c r="H106" s="4"/>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E106" s="5"/>
+      <c r="F106" s="5"/>
+      <c r="G106" s="5"/>
+      <c r="H106" s="5"/>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B107" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C107" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D107">
         <v>1</v>
       </c>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E107" s="5"/>
+      <c r="F107" s="5"/>
+      <c r="G107" s="5"/>
+      <c r="H107" s="5"/>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="B108" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C108" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D108">
         <v>8</v>
       </c>
-      <c r="E108" s="4"/>
-      <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
-      <c r="H108" s="4"/>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E108" s="5"/>
+      <c r="F108" s="5"/>
+      <c r="G108" s="5"/>
+      <c r="H108" s="5"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="B109" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C109" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D109">
         <v>0</v>
       </c>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
-      <c r="H109" s="4"/>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
+      <c r="G109" s="5"/>
+      <c r="H109" s="5"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="B110" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C110" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D110">
         <v>7</v>
       </c>
-      <c r="E110" s="4"/>
-      <c r="F110" s="4"/>
-      <c r="G110" s="4"/>
-      <c r="H110" s="4"/>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
+      <c r="G110" s="5"/>
+      <c r="H110" s="5"/>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B111" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C111" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
-      <c r="E111" s="4"/>
-      <c r="F111" s="4"/>
-      <c r="G111" s="4"/>
-      <c r="H111" s="4"/>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
+      <c r="G111" s="5"/>
+      <c r="H111" s="5"/>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B112" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C112" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D112">
         <v>2</v>
       </c>
-      <c r="E112" s="4"/>
-      <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
-      <c r="H112" s="4"/>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" s="5"/>
+      <c r="H112" s="5"/>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B113" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C113" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D113">
         <v>1</v>
       </c>
-      <c r="E113" s="4"/>
-      <c r="F113" s="4"/>
-      <c r="G113" s="4"/>
-      <c r="H113" s="4"/>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
+      <c r="G113" s="5"/>
+      <c r="H113" s="5"/>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B114" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C114" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D114">
         <v>1</v>
       </c>
-      <c r="E114" s="4"/>
-      <c r="F114" s="4"/>
-      <c r="G114" s="4"/>
-      <c r="H114" s="4"/>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
+      <c r="G114" s="5"/>
+      <c r="H114" s="5"/>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B115" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C115" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D115">
         <v>2</v>
       </c>
-      <c r="E115" s="4"/>
-      <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
-      <c r="H115" s="4"/>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="5"/>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B116" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C116" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D116">
         <v>2</v>
       </c>
-      <c r="E116" s="4"/>
-      <c r="F116" s="4"/>
-      <c r="G116" s="4"/>
-      <c r="H116" s="4"/>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5"/>
+      <c r="H116" s="5"/>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B117" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C117" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D117">
         <v>1</v>
       </c>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
-      <c r="G117" s="4"/>
-      <c r="H117" s="4"/>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="5"/>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B118" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C118" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D118">
         <v>3</v>
       </c>
-      <c r="E118" s="4"/>
-      <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
-      <c r="H118" s="4"/>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5"/>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B119" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C119" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D119">
         <v>2</v>
       </c>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
-      <c r="H119" s="4"/>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="5"/>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B120" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C120" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D120">
         <v>1</v>
       </c>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
-      <c r="H120" s="4"/>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5"/>
+      <c r="H120" s="5"/>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B121" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C121" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D121">
         <v>5</v>
       </c>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5"/>
+      <c r="H121" s="5"/>
       <c r="J121" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B122" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C122" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D122">
         <v>3</v>
       </c>
-      <c r="E122" s="4"/>
-      <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
-      <c r="H122" s="4"/>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5"/>
+      <c r="H122" s="5"/>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B123" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="C123" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D123">
         <v>3</v>
       </c>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
-      <c r="H123" s="4"/>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5"/>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B124" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="C124" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D124">
         <v>2</v>
       </c>
-      <c r="E124" s="4"/>
-      <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
-      <c r="H124" s="4"/>
+      <c r="E124" s="5"/>
+      <c r="F124" s="5"/>
+      <c r="G124" s="5"/>
+      <c r="H124" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J124" xr:uid="{8517A870-A2C1-9449-9CD8-8187ABBC08FC}"/>
+  <autoFilter ref="A1:J124"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding forcenew attributes to the site (#110)
</commit_message>
<xml_diff>
--- a/scripts/templates/cx-as-code-spreadsheet-template.xlsx
+++ b/scripts/templates/cx-as-code-spreadsheet-template.xlsx
@@ -1,56 +1,52 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ascheble/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8076B3B-A0D9-3942-A179-08CFA0AF627B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{166D1F10-E3AB-E94C-B675-684CCFA97A59}"/>
+    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680"/>
   </bookViews>
   <sheets>
-    <sheet name="resources" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="resources" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">resources!$A$1:$J$124</definedName>
+    <definedName name="_xlnm._FilterDatabase">resources!$A$1:$J$124</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="246">
   <si>
+    <t>GUI Menu Path</t>
+  </si>
+  <si>
     <t>CX as Code Resource Type</t>
   </si>
   <si>
     <t>Division-aware</t>
   </si>
   <si>
-    <t>Possible Dependencies</t>
+    <t>Dependencies</t>
+  </si>
+  <si>
+    <t>In/out of scope</t>
+  </si>
+  <si>
+    <t>Shared?</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Repo/Project/Folder</t>
+  </si>
+  <si>
+    <t>Transform type</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
   <si>
     <t>User Management &gt; ACD Skills and Languages &gt; Languages</t>
@@ -759,61 +755,47 @@
   </si>
   <si>
     <t>genesyscloud_webdeployments_deployment</t>
-  </si>
-  <si>
-    <t>GUI Menu Path</t>
-  </si>
-  <si>
-    <t>Repo/Project/Folder</t>
-  </si>
-  <si>
-    <t>Transform type</t>
-  </si>
-  <si>
-    <t>Shared?</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>In/out of scope</t>
-  </si>
-  <si>
-    <t>Notes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -844,13 +826,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1164,2269 +1146,2268 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444CE756-FC6B-BB41-9CFA-B458F0085971}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J124"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="73.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="67" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="11" max="11" width="2" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D16">
         <v>3</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>2</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C22" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D24">
         <v>1</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D27">
         <v>8</v>
       </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C30" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>13</v>
       </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D32">
         <v>3</v>
       </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C33" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C35" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D36">
         <v>1</v>
       </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D37">
         <v>3</v>
       </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C38" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D39">
         <v>2</v>
       </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D40">
         <v>0</v>
       </c>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D41">
         <v>3</v>
       </c>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D42">
         <v>2</v>
       </c>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B43" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D43">
         <v>2</v>
       </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C44" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D44">
         <v>2</v>
       </c>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C45" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D45">
         <v>0</v>
       </c>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D46">
         <v>0</v>
       </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C47" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D47">
         <v>1</v>
       </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C48" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C49" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C50" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D50">
         <v>0</v>
       </c>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C51" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D51">
         <v>0</v>
       </c>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C52" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C53" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D53">
         <v>0</v>
       </c>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C54" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D54">
         <v>0</v>
       </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B55" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C55" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D55">
         <v>0</v>
       </c>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B56" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C56" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D56">
         <v>2</v>
       </c>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="C57" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D57">
         <v>0</v>
       </c>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B58" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B59" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C59" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D59">
         <v>0</v>
       </c>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B60" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C60" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D60">
         <v>0</v>
       </c>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C61" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D61">
         <v>0</v>
       </c>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B62" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D62">
         <v>0</v>
       </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C63" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D63">
         <v>0</v>
       </c>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C64" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D64">
         <v>1</v>
       </c>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B65" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C65" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D65">
         <v>1</v>
       </c>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="5"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B66" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C66" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D66">
         <v>2</v>
       </c>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B67" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C67" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D67">
         <v>5</v>
       </c>
-      <c r="E67" s="4"/>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C68" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D68">
         <v>0</v>
       </c>
-      <c r="E68" s="4"/>
-      <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B69" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C69" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D69">
         <v>0</v>
       </c>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B70" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C70" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D71">
         <v>0</v>
       </c>
-      <c r="E71" s="4"/>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B72" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C72" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D72">
         <v>0</v>
       </c>
-      <c r="E72" s="4"/>
-      <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B73" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C73" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D73">
         <v>0</v>
       </c>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="5"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C74" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D74">
         <v>1</v>
       </c>
-      <c r="E74" s="4"/>
-      <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B75" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C75" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D75">
         <v>1</v>
       </c>
-      <c r="E75" s="4"/>
-      <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
-      <c r="H75" s="4"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B76" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C76" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D76">
         <v>2</v>
       </c>
-      <c r="E76" s="4"/>
-      <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
-      <c r="H76" s="4"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B77" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C77" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D77">
         <v>0</v>
       </c>
-      <c r="E77" s="4"/>
-      <c r="F77" s="4"/>
-      <c r="G77" s="4"/>
-      <c r="H77" s="4"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5"/>
+      <c r="H77" s="5"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B78" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C78" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D78">
         <v>1</v>
       </c>
-      <c r="E78" s="4"/>
-      <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
-      <c r="H78" s="4"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5"/>
+      <c r="H78" s="5"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B79" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C79" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D79">
         <v>3</v>
       </c>
-      <c r="E79" s="4"/>
-      <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B80" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C80" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D80">
         <v>0</v>
       </c>
-      <c r="E80" s="4"/>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B81" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C81" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D81">
         <v>1</v>
       </c>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
-      <c r="H81" s="4"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B82" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C82" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D82">
         <v>0</v>
       </c>
-      <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
-      <c r="G82" s="4"/>
-      <c r="H82" s="4"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B83" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C83" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D83">
         <v>0</v>
       </c>
-      <c r="E83" s="4"/>
-      <c r="F83" s="4"/>
-      <c r="G83" s="4"/>
-      <c r="H83" s="4"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B84" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C84" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D84">
         <v>1</v>
       </c>
-      <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
-      <c r="G84" s="4"/>
-      <c r="H84" s="4"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B85" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C85" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D85">
         <v>11</v>
       </c>
-      <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
-      <c r="H85" s="4"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B86" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C86" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D86">
         <v>5</v>
       </c>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-      <c r="H86" s="4"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5"/>
+      <c r="H86" s="5"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B87" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C87" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D87">
         <v>2</v>
       </c>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
-      <c r="H87" s="4"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
+      <c r="H87" s="5"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B88" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C88" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D88">
         <v>2</v>
       </c>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
-      <c r="G88" s="4"/>
-      <c r="H88" s="4"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="5"/>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B89" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C89" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D89">
         <v>2</v>
       </c>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
-      <c r="H89" s="4"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B90" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C90" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D90">
         <v>1</v>
       </c>
-      <c r="E90" s="4"/>
-      <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
-      <c r="H90" s="4"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B91" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C91" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D91">
         <v>1</v>
       </c>
-      <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
-      <c r="H91" s="4"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B92" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C92" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D92">
         <v>0</v>
       </c>
-      <c r="E92" s="4"/>
-      <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
-      <c r="H92" s="4"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B93" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C93" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D93">
         <v>9</v>
       </c>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
-      <c r="H93" s="4"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B94" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C94" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D94">
         <v>4</v>
       </c>
-      <c r="E94" s="4"/>
-      <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
-      <c r="H94" s="4"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B95" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C95" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D95">
         <v>1</v>
       </c>
-      <c r="E95" s="4"/>
-      <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
-      <c r="H95" s="4"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B96" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C96" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D96">
         <v>0</v>
       </c>
-      <c r="E96" s="4"/>
-      <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
-      <c r="H96" s="4"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B97" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C97" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D97">
         <v>1</v>
       </c>
-      <c r="E97" s="4"/>
-      <c r="F97" s="4"/>
-      <c r="G97" s="4"/>
-      <c r="H97" s="4"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B98" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C98" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D98">
         <v>1</v>
       </c>
-      <c r="E98" s="4"/>
-      <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
-      <c r="H98" s="4"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5"/>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B99" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C99" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D99">
         <v>2</v>
       </c>
-      <c r="E99" s="4"/>
-      <c r="F99" s="4"/>
-      <c r="G99" s="4"/>
-      <c r="H99" s="4"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B100" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C100" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D100">
         <v>1</v>
       </c>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
-      <c r="H100" s="4"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5"/>
+      <c r="H100" s="5"/>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B101" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C101" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D101">
         <v>5</v>
       </c>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
-      <c r="H101" s="4"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
+      <c r="G101" s="5"/>
+      <c r="H101" s="5"/>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B102" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C102" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D102">
         <v>0</v>
       </c>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
-      <c r="H102" s="4"/>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E102" s="5"/>
+      <c r="F102" s="5"/>
+      <c r="G102" s="5"/>
+      <c r="H102" s="5"/>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B103" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C103" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D103">
         <v>0</v>
       </c>
-      <c r="E103" s="4"/>
-      <c r="F103" s="4"/>
-      <c r="G103" s="4"/>
-      <c r="H103" s="4"/>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E103" s="5"/>
+      <c r="F103" s="5"/>
+      <c r="G103" s="5"/>
+      <c r="H103" s="5"/>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B104" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C104" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D104">
         <v>0</v>
       </c>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
-      <c r="H104" s="4"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E104" s="5"/>
+      <c r="F104" s="5"/>
+      <c r="G104" s="5"/>
+      <c r="H104" s="5"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B105" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C105" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D105">
         <v>0</v>
       </c>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
-      <c r="G105" s="4"/>
-      <c r="H105" s="4"/>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
+      <c r="G105" s="5"/>
+      <c r="H105" s="5"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="B106" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C106" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D106">
         <v>1</v>
       </c>
-      <c r="E106" s="4"/>
-      <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
-      <c r="H106" s="4"/>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E106" s="5"/>
+      <c r="F106" s="5"/>
+      <c r="G106" s="5"/>
+      <c r="H106" s="5"/>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B107" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C107" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D107">
         <v>1</v>
       </c>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E107" s="5"/>
+      <c r="F107" s="5"/>
+      <c r="G107" s="5"/>
+      <c r="H107" s="5"/>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="B108" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C108" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D108">
         <v>8</v>
       </c>
-      <c r="E108" s="4"/>
-      <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
-      <c r="H108" s="4"/>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E108" s="5"/>
+      <c r="F108" s="5"/>
+      <c r="G108" s="5"/>
+      <c r="H108" s="5"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="B109" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C109" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D109">
         <v>0</v>
       </c>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
-      <c r="H109" s="4"/>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
+      <c r="G109" s="5"/>
+      <c r="H109" s="5"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="B110" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C110" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D110">
         <v>7</v>
       </c>
-      <c r="E110" s="4"/>
-      <c r="F110" s="4"/>
-      <c r="G110" s="4"/>
-      <c r="H110" s="4"/>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
+      <c r="G110" s="5"/>
+      <c r="H110" s="5"/>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B111" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C111" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
-      <c r="E111" s="4"/>
-      <c r="F111" s="4"/>
-      <c r="G111" s="4"/>
-      <c r="H111" s="4"/>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
+      <c r="G111" s="5"/>
+      <c r="H111" s="5"/>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B112" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C112" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D112">
         <v>2</v>
       </c>
-      <c r="E112" s="4"/>
-      <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
-      <c r="H112" s="4"/>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" s="5"/>
+      <c r="H112" s="5"/>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B113" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C113" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D113">
         <v>1</v>
       </c>
-      <c r="E113" s="4"/>
-      <c r="F113" s="4"/>
-      <c r="G113" s="4"/>
-      <c r="H113" s="4"/>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
+      <c r="G113" s="5"/>
+      <c r="H113" s="5"/>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B114" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C114" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D114">
         <v>1</v>
       </c>
-      <c r="E114" s="4"/>
-      <c r="F114" s="4"/>
-      <c r="G114" s="4"/>
-      <c r="H114" s="4"/>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
+      <c r="G114" s="5"/>
+      <c r="H114" s="5"/>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B115" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C115" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D115">
         <v>2</v>
       </c>
-      <c r="E115" s="4"/>
-      <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
-      <c r="H115" s="4"/>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="5"/>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B116" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C116" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D116">
         <v>2</v>
       </c>
-      <c r="E116" s="4"/>
-      <c r="F116" s="4"/>
-      <c r="G116" s="4"/>
-      <c r="H116" s="4"/>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5"/>
+      <c r="H116" s="5"/>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B117" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C117" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D117">
         <v>1</v>
       </c>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
-      <c r="G117" s="4"/>
-      <c r="H117" s="4"/>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="5"/>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B118" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C118" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D118">
         <v>3</v>
       </c>
-      <c r="E118" s="4"/>
-      <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
-      <c r="H118" s="4"/>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5"/>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B119" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C119" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D119">
         <v>2</v>
       </c>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
-      <c r="H119" s="4"/>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="5"/>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B120" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C120" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D120">
         <v>1</v>
       </c>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
-      <c r="H120" s="4"/>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5"/>
+      <c r="H120" s="5"/>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B121" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C121" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D121">
         <v>5</v>
       </c>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5"/>
+      <c r="H121" s="5"/>
       <c r="J121" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B122" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C122" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D122">
         <v>3</v>
       </c>
-      <c r="E122" s="4"/>
-      <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
-      <c r="H122" s="4"/>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5"/>
+      <c r="H122" s="5"/>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B123" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="C123" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D123">
         <v>3</v>
       </c>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
-      <c r="H123" s="4"/>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5"/>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B124" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="C124" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D124">
         <v>2</v>
       </c>
-      <c r="E124" s="4"/>
-      <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
-      <c r="H124" s="4"/>
+      <c r="E124" s="5"/>
+      <c r="F124" s="5"/>
+      <c r="G124" s="5"/>
+      <c r="H124" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J124" xr:uid="{8517A870-A2C1-9449-9CD8-8187ABBC08FC}"/>
+  <autoFilter ref="A1:J124"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>